<commit_message>
Build q2436 Airflow Windows reproduction
</commit_message>
<xml_diff>
--- a/task/任务规格转化.xlsx
+++ b/task/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R05c0ab96bb024467"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="Rdf6064de5e76444c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,7 +13,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="4">
+  <x:fonts count="2">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -24,19 +24,8 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
-    <x:font>
-      <x:sz val="10"/>
-      <x:color rgb="FF243746"/>
-      <x:name val="Carlito"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="10"/>
-      <x:color rgb="FF243746"/>
-      <x:name val="Carlito"/>
-    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="3">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -45,101 +34,48 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF34546F"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFFFFF"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE8F0F5"/>
+        <x:fgColor rgb="FF3A5668"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="3">
+  <x:borders count="2">
     <x:border/>
     <x:border>
-      <x:left style="thin">
-        <x:color rgb="FFCCD6DF"/>
-      </x:left>
-      <x:right style="thin">
-        <x:color rgb="FFCCD6DF"/>
-      </x:right>
-      <x:top style="thin">
-        <x:color rgb="FFCCD6DF"/>
-      </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FFCCD6DF"/>
-      </x:bottom>
-    </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color rgb="FFD8E0E7"/>
-      </x:left>
-      <x:right style="thin">
-        <x:color rgb="FFD8E0E7"/>
-      </x:right>
-      <x:top style="thin">
-        <x:color rgb="FFD8E0E7"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FFD8E0E7"/>
+        <x:color rgb="FFD7E1E7"/>
       </x:bottom>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="15">
+  <x:cellXfs count="9">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TaskSpecTable" displayName="TaskSpecTable" ref="A1:B15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="2">
-    <x:tableColumn id="1" name="模块"/>
-    <x:tableColumn id="2" name="规格内容"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -337,134 +273,147 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="36" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="138" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="132" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="6" t="str">
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
+      <x:c r="A1" s="8" t="str">
         <x:v>模块</x:v>
       </x:c>
-      <x:c r="B1" s="6" t="str">
+      <x:c r="B1" s="8" t="str">
         <x:v>规格内容</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="31" customHeight="1">
-      <x:c r="A2" s="14" t="str">
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="5" t="str">
         <x:v>任务ID</x:v>
       </x:c>
-      <x:c r="B2" s="12" t="str">
-        <x:v>airflow_moderation_failure_pause_replay</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="57" customHeight="1">
-      <x:c r="A3" s="14" t="str">
+      <x:c r="B2" s="5" t="str">
+        <x:v>airflow_moderation_pause_handover</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="5" t="str">
         <x:v>主软件</x:v>
       </x:c>
-      <x:c r="B3" s="12" t="str">
-        <x:v>ApacheAirflow2.10.5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="44" customHeight="1">
-      <x:c r="A4" s="14" t="str">
+      <x:c r="B3" s="5" t="str">
+        <x:v>Apache Airflow</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="5" t="str">
         <x:v>辅助工具</x:v>
       </x:c>
-      <x:c r="B4" s="12" t="str">
-        <x:v>主软件为ApacheAirflow2.10.5。Windows11主机通过WSL2运行官方支持的Linux环境，不能写成原生Windows运行。 安装阶段可以联网取得主软件和锁定依赖，正式复现只读取题目输入并使用本机回环连接。辅助工具为PowerShell、Git和文本编辑器；公开仓库不包含凭据，许可按各软件原许可执行。 建议准备2核CPU、4GB内存和2GB可用磁盘。权限限制为输入目录只读，程序只能写入指定工作目录；单次执行超时为15分钟，人工完成预计4至8小时。 主要风险是复用旧元数据库造成隐藏DagRun、把owner=scheduler误解为已启动Scheduler、在解封时清除失败历史，或让CSV结果替代Airflow表记录；</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="44" customHeight="1">
-      <x:c r="A5" s="14" t="str">
+      <x:c r="B4" s="5" t="str">
+        <x:v>WSL2、Ubuntu24.04、Python3.11、PowerShell7、SQLite查看工具和文本编辑器</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="5" t="str">
         <x:v>输入来源</x:v>
       </x:c>
-      <x:c r="B5" s="12" t="str">
-        <x:v>依据内容平台审核结果发布保护场景编写的离线策略、事件时间线和阈值禁用starter，不含真实用户、审核文本或生产日志</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="44" customHeight="1">
-      <x:c r="A6" s="14" t="str">
+      <x:c r="B5" s="5" t="str">
+        <x:v>内容平台发布保障组提供的暂停策略、历史运行时间线和当前DAG</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="5" t="str">
         <x:v>输入获取方式</x:v>
       </x:c>
-      <x:c r="B6" s="12" t="str">
-        <x:v>随输入数据包.zip离线提供；解压后从input_data/README.md进入，四个输入文件保持只读</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="70" customHeight="1">
-      <x:c r="A7" s="14" t="str">
+      <x:c r="B6" s="5" t="str">
+        <x:v>从输入数据包解压到本地只读目录</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="5" t="str">
         <x:v>原始输入文件</x:v>
       </x:c>
-      <x:c r="B7" s="12" t="str">
-        <x:v>输入数据包解压目录保持只读，所有生成内容写入指定工作目录</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="83" customHeight="1">
-      <x:c r="A8" s="14" t="str">
+      <x:c r="B7" s="5" t="str">
+        <x:v>input_data/pause_policy.json、incident_timeline.csv、starter/broken_moderation_feed.py和README.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="5" t="str">
         <x:v>目标输出文件</x:v>
       </x:c>
-      <x:c r="B8" s="12" t="str">
-        <x:v>output/README.md；output/dags/moderation_feed_publish_guard.py；output/solution/metastore_replayer.py；output/tools/run_reference.py；output/tests/test_results.py；output/results下六份证据文件</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="44" customHeight="1">
-      <x:c r="A9" s="14" t="str">
+      <x:c r="B8" s="5" t="str">
+        <x:v>output/dags修复版DAG、output/tools审计入口、output/results四份结构化结果和output/HANDOVER.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="5" t="str">
         <x:v>核心操作链</x:v>
       </x:c>
-      <x:c r="B9" s="12" t="str">
-        <x:v>核对input_data/下四个文件的相对路径、事件表头、sequence连续性、event_id唯一性、终态与策略字段。→解析starter/broken_moderation_feed.py，确认待修复缺陷是连续失败阈值被禁用且原任务图仍完整。→把修复后的DAG写入output/dags/moderation_feed_publish_guard.py，使调度属性、任务边和阈值与pause_policy.json一致。→将每个DAGRUN事件作为manual且external_trigger=true的真实DagRun写入隔离元数据库，保留logical_date和终态。→调用Airflow连续失败检查处理failed运行，通过DagModel.set_is_paused(false)执行管理员解封并保留全部运行历史。→查询DagRun历史后缀、DagModel暂停开关和Log表paused行，按事件前后状态推导连续失败数、日志增量与verdict。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="44" customHeight="1">
-      <x:c r="A10" s="14" t="str">
-        <x:v>数据范围</x:v>
-      </x:c>
-      <x:c r="B10" s="12" t="str">
-        <x:v>14个事件，其中12个DagRun和2个管理员解封；4个success、8个failed；当前阈值3；真实paused日志2行</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="44" customHeight="1">
-      <x:c r="A11" s="14" t="str">
-        <x:v>精度要求</x:v>
-      </x:c>
-      <x:c r="B11" s="12" t="str">
-        <x:v>sequence、event_id、run_id、logical_date、终态、任务和依赖边精确比较；暂停轨迹按整数后缀和布尔值比较；非业务日志ID与时间不评分</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="57" customHeight="1">
-      <x:c r="A12" s="14" t="str">
-        <x:v>裁决原则</x:v>
-      </x:c>
-      <x:c r="B12" s="12" t="str">
-        <x:v>阈值以pause_policy.json为来源；连续失败数以logical_date倒序的真实DagRun后缀为准；解封只改暂停开关；owner=scheduler是Airflow方法写入值而非进程运行校核</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="44" customHeight="1">
-      <x:c r="A13" s="14" t="str">
+      <x:c r="B9" s="5" t="str">
+        <x:v>核对策略与当前DAG→恢复失败阈值→DagBag加载→迁移元数据库→同步DAG→处理运行时间线→执行状态更新→导出暂停轨迹→完成交接</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="5" t="str">
+        <x:v>DAG配置</x:v>
+      </x:c>
+      <x:c r="B10" s="5" t="str">
+        <x:v>dag_id、schedule、catchup、max_active_runs、is_paused_upon_creation、任务集合、依赖边和失败阈值均来自pause_policy.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="5" t="str">
+        <x:v>运行落库</x:v>
+      </x:c>
+      <x:c r="B11" s="5" t="str">
+        <x:v>DAGRUN事件创建manual DagRun并保留run_id、logical_date和终态，external_trigger为true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="5" t="str">
+        <x:v>暂停判断</x:v>
+      </x:c>
+      <x:c r="B12" s="5" t="str">
+        <x:v>运行终态由DagRun.update_state确定，自动暂停以DagModel状态和Airflow Log中的paused事件为证据</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="5" t="str">
+        <x:v>管理员解封</x:v>
+      </x:c>
+      <x:c r="B13" s="5" t="str">
+        <x:v>ADMIN_UNPAUSE只更新DagModel暂停状态，既有DagRun和失败后缀保持不变</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="5" t="str">
+        <x:v>交付结果</x:v>
+      </x:c>
+      <x:c r="B14" s="5" t="str">
+        <x:v>事件台账、DagRun历史、DAG快照和暂停事件来自同一Airflow元数据库并可相互核对</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="5" t="str">
         <x:v>完成条件</x:v>
       </x:c>
-      <x:c r="B13" s="12" t="str">
-        <x:v>DAG通过DagBag加载并运行目标任务语义，输出与Reference一致</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="57" customHeight="1">
-      <x:c r="A14" s="14" t="str">
+      <x:c r="B15" s="5" t="str">
+        <x:v>DAG通过DagBag加载，策略恢复，时间线完整落库，自动暂停和解封轨迹符合输入顺序，交接说明与结果一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="5" t="str">
         <x:v>可验证点</x:v>
       </x:c>
-      <x:c r="B14" s="12" t="str">
-        <x:v>Windows主机与WSL2版本、DagBag导入、dag_run和dag表、Log原始行、event_ledger输入投影、dagrun_history、DagModel快照、SerializedDAG、validation checks和两次空库复演</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="44" customHeight="1">
-      <x:c r="A15" s="14" t="str">
+      <x:c r="B16" s="5" t="str">
+        <x:v>DAG对象属性、任务边、DagRun主键与终态、DagModel暂停状态、Log中的paused事件、失败后缀及四份结果的一致性</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="6" t="str">
         <x:v>不适合作为评分点的内容</x:v>
       </x:c>
-      <x:c r="B15" s="12" t="str">
-        <x:v>ORM会话拆分；函数名；测试数量；validation checks数量；JSON键序；CSV非主键行序；Log内部id和dttm；临时目录名称；绝对路径</x:v>
+      <x:c r="B17" s="6" t="str">
+        <x:v>Python排版、函数名、Airflow内部日志ID、日志时间、JSON键序、CSV非主键行序和交接说明措辞</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R227bad9b45344bd5"/>
-  </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>